<commit_message>
Rent Cars: add 3 cars (CX-90, GV70, GV80), user revisions, split 2 maybes; back up model
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_files/Rent_Cars_Fleet_Model.xlsx
+++ b/project_files/Rent_Cars_Fleet_Model.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="118">
   <si>
     <t>Vehicle</t>
   </si>
@@ -120,6 +120,24 @@
     <t>5-Yr Cumulative Profit</t>
   </si>
   <si>
+    <t>Mazda CX-90</t>
+  </si>
+  <si>
+    <t>Luxury Family SUV</t>
+  </si>
+  <si>
+    <t>Genesis GV70</t>
+  </si>
+  <si>
+    <t>Luxury Compact SUV</t>
+  </si>
+  <si>
+    <t>Genesis GV80</t>
+  </si>
+  <si>
+    <t>Luxury 3-Row SUV</t>
+  </si>
+  <si>
     <t>Porsche 911 Carrera Cabriolet</t>
   </si>
   <si>
@@ -153,9 +171,6 @@
     <t>Luxury Adventure</t>
   </si>
   <si>
-    <t>Lotus Emira (V6 auto)</t>
-  </si>
-  <si>
     <t>Chevrolet C7 Corvette</t>
   </si>
   <si>
@@ -168,7 +183,7 @@
     <t>Off-Road</t>
   </si>
   <si>
-    <t>Toyota Tacoma</t>
+    <t>Ram Rebel</t>
   </si>
   <si>
     <t>Adventure Truck</t>
@@ -183,18 +198,21 @@
     <t>Lexus GX 550</t>
   </si>
   <si>
-    <t>Luxury Family SUV</t>
-  </si>
-  <si>
-    <t>Toyota Supra</t>
-  </si>
-  <si>
     <t>Lexus LX 600</t>
   </si>
   <si>
     <t>Full-Size Luxury</t>
   </si>
   <si>
+    <t>FLEET TOTAL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>MAYBES — UNDER CONSIDERATION  (not included in the Fleet Total above)</t>
+  </si>
+  <si>
     <t>Ineos Grenadier</t>
   </si>
   <si>
@@ -207,13 +225,7 @@
     <t>Ski / Family Hauler</t>
   </si>
   <si>
-    <t>FLEET TOTAL</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>FLEET SUMMARY (16 vehicles)</t>
+    <t>FLEET SUMMARY (15 confirmed vehicles — maybes excluded)</t>
   </si>
   <si>
     <t>Total Purchase Price</t>
@@ -282,13 +294,28 @@
     <t>Rent direct through own website. Based in Denver near the I-70 corridor.</t>
   </si>
   <si>
+    <t>Numbers source</t>
+  </si>
+  <si>
+    <t>Confirmed-fleet inputs (price/rate/days/residual/etc.) reflect your revised values. The 3 new cars (Mazda CX-90, Genesis GV70, Genesis GV80) use seeded estimates — verify Genesis residuals especially.</t>
+  </si>
+  <si>
+    <t>MAYBES</t>
+  </si>
+  <si>
+    <t>Under consideration</t>
+  </si>
+  <si>
+    <t>Ineos Grenadier and Mercedes R-Class are shown below the Fleet Total and are EXCLUDED from all totals/summary. Move them up into CONFIRMED if you commit.</t>
+  </si>
+  <si>
     <t>VEHICLE KIT (one-time, amortized over 5 yrs)</t>
   </si>
   <si>
     <t>Sports / exotic</t>
   </si>
   <si>
-    <t>NOW carry tires: winter $1,600 + summer $1,400. No roof box / fridge / camping.</t>
+    <t>Carry tires only: winter $1,600 + summer $1,400. No roof box / fridge / camping.</t>
   </si>
   <si>
     <t>SUV / truck</t>
@@ -306,39 +333,24 @@
     <t>Camping pack</t>
   </si>
   <si>
-    <t>Optional add-on — carried on SUVs &amp; vans only. Generates upsell revenue (see below).</t>
+    <t>Optional add-on — carried on SUVs &amp; vans only. Generates upsell revenue.</t>
   </si>
   <si>
     <t>TIRE REFRESH (ongoing)</t>
   </si>
   <si>
-    <t>= (Winter + Summer tires) ÷ 3-yr tire life. Funds replacement as studded/perf tires wear.</t>
-  </si>
-  <si>
-    <t>Applies</t>
-  </si>
-  <si>
-    <t>Hits BOTH during-loan and post-loan net — tires keep wearing after the car is paid off.</t>
+    <t>= (Winter + Summer tires) ÷ 3-yr tire life. Hits BOTH during-loan and post-loan net.</t>
   </si>
   <si>
     <t>CAMPING UPSELL REVENUE</t>
   </si>
   <si>
-    <t>$35/day add-on when a guest rents the camping pack</t>
-  </si>
-  <si>
-    <t>25% of rental days include the camping pack (SUVs &amp; vans)</t>
-  </si>
-  <si>
-    <t>= Rental Days/Yr × Attach % × Camp $/Day. Added into Gross Revenue.</t>
+    <t>= Rental Days/Yr × 25% attach × $35/day. Added into Gross Revenue (SUVs &amp; vans).</t>
   </si>
   <si>
     <t>5-YEAR OUTPUTS</t>
   </si>
   <si>
-    <t>Resale as % of purchase price by type. Porsche/Toyota/Lexus hold value; 356 appreciates (105%); R-Class weakest (60%).</t>
-  </si>
-  <si>
     <t>= Purchase Price × Residual %</t>
   </si>
   <si>
@@ -355,12 +367,6 @@
   </si>
   <si>
     <t>Prices, rates, days/mo, kit costs, camp attach %, residual %, miles/day all recalc automatically.</t>
-  </si>
-  <si>
-    <t>Under-consideration cars</t>
-  </si>
-  <si>
-    <t>Lexus LX 600, Ineos Grenadier, Mercedes R-Class still "under consideration" — included for comparison.</t>
   </si>
 </sst>
 </file>
@@ -372,7 +378,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -390,6 +396,10 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF9C5700"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
     </font>
     <font>
@@ -397,7 +407,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -414,6 +424,16 @@
         <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDF2E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -427,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -458,13 +478,24 @@
     <xf numFmtId="3" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -806,7 +837,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AI18"/>
+  <dimension ref="A1:AI21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -941,7 +972,7 @@
         <v>36</v>
       </c>
       <c r="C2" s="1">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
@@ -959,19 +990,19 @@
         <f>PMT(F2/12,G2*12,-E2)*12</f>
       </c>
       <c r="I2" s="1">
+        <v>2200</v>
+      </c>
+      <c r="J2" s="1">
         <v>1600</v>
       </c>
-      <c r="J2" s="1">
-        <v>1400</v>
-      </c>
       <c r="K2" s="1">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L2" s="1">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="M2" s="1">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="N2" s="1">
         <f>SUM(I2:M2)</f>
@@ -983,19 +1014,19 @@
         <f>(I2+J2)/3</f>
       </c>
       <c r="Q2" s="1">
+        <v>2000</v>
+      </c>
+      <c r="R2" s="1">
         <v>2500</v>
       </c>
-      <c r="R2" s="1">
-        <v>5000</v>
-      </c>
       <c r="S2" s="1">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="T2" s="1">
-        <v>335</v>
+        <v>160</v>
       </c>
       <c r="U2" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="V2" s="3">
         <f>U2*12</f>
@@ -1004,10 +1035,10 @@
         <f>T2*V2</f>
       </c>
       <c r="X2" s="1">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="Y2" s="2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Z2" s="1">
         <f>V2*Y2*X2</f>
@@ -1025,13 +1056,13 @@
         <f>AA2-AB2-P2-Q2-R2-S2</f>
       </c>
       <c r="AE2" s="2">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="AF2" s="1">
         <f>C2*AE2</f>
       </c>
       <c r="AG2" s="3">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="AH2" s="3">
         <f>V2*AG2*5</f>
@@ -1048,7 +1079,7 @@
         <v>38</v>
       </c>
       <c r="C3" s="1">
-        <v>45000</v>
+        <v>58000</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
@@ -1066,19 +1097,19 @@
         <f>PMT(F3/12,G3*12,-E3)*12</f>
       </c>
       <c r="I3" s="1">
+        <v>2200</v>
+      </c>
+      <c r="J3" s="1">
         <v>1600</v>
       </c>
-      <c r="J3" s="1">
-        <v>1400</v>
-      </c>
       <c r="K3" s="1">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L3" s="1">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="M3" s="1">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="N3" s="1">
         <f>SUM(I3:M3)</f>
@@ -1090,19 +1121,19 @@
         <f>(I3+J3)/3</f>
       </c>
       <c r="Q3" s="1">
-        <v>2500</v>
+        <v>2200</v>
       </c>
       <c r="R3" s="1">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="S3" s="1">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="T3" s="1">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="U3" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="V3" s="3">
         <f>U3*12</f>
@@ -1111,10 +1142,10 @@
         <f>T3*V3</f>
       </c>
       <c r="X3" s="1">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="Y3" s="2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Z3" s="1">
         <f>V3*Y3*X3</f>
@@ -1132,13 +1163,13 @@
         <f>AA3-AB3-P3-Q3-R3-S3</f>
       </c>
       <c r="AE3" s="2">
-        <v>1.05</v>
+        <v>0.62</v>
       </c>
       <c r="AF3" s="1">
         <f>C3*AE3</f>
       </c>
       <c r="AG3" s="3">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="AH3" s="3">
         <f>V3*AG3*5</f>
@@ -1155,7 +1186,7 @@
         <v>40</v>
       </c>
       <c r="C4" s="1">
-        <v>45000</v>
+        <v>70000</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
@@ -1173,10 +1204,10 @@
         <f>PMT(F4/12,G4*12,-E4)*12</f>
       </c>
       <c r="I4" s="1">
-        <v>1400</v>
+        <v>2200</v>
       </c>
       <c r="J4" s="1">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="K4" s="1">
         <v>1000</v>
@@ -1197,19 +1228,19 @@
         <f>(I4+J4)/3</f>
       </c>
       <c r="Q4" s="1">
-        <v>1800</v>
+        <v>2400</v>
       </c>
       <c r="R4" s="1">
-        <v>2500</v>
+        <v>3200</v>
       </c>
       <c r="S4" s="1">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="T4" s="1">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="U4" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V4" s="3">
         <f>U4*12</f>
@@ -1245,7 +1276,7 @@
         <f>C4*AE4</f>
       </c>
       <c r="AG4" s="3">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="AH4" s="3">
         <f>V4*AG4*5</f>
@@ -1262,7 +1293,7 @@
         <v>42</v>
       </c>
       <c r="C5" s="1">
-        <v>32000</v>
+        <v>60000</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
@@ -1304,19 +1335,19 @@
         <f>(I5+J5)/3</f>
       </c>
       <c r="Q5" s="1">
-        <v>1800</v>
+        <v>2500</v>
       </c>
       <c r="R5" s="1">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="S5" s="1">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="T5" s="1">
-        <v>120</v>
+        <v>335</v>
       </c>
       <c r="U5" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V5" s="3">
         <f>U5*12</f>
@@ -1346,7 +1377,7 @@
         <f>AA5-AB5-P5-Q5-R5-S5</f>
       </c>
       <c r="AE5" s="2">
-        <v>0.68</v>
+        <v>0.85</v>
       </c>
       <c r="AF5" s="1">
         <f>C5*AE5</f>
@@ -1366,10 +1397,10 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C6" s="1">
-        <v>75000</v>
+        <v>45000</v>
       </c>
       <c r="D6" s="1">
         <v>0</v>
@@ -1414,16 +1445,16 @@
         <v>2500</v>
       </c>
       <c r="R6" s="1">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="S6" s="1">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="T6" s="1">
-        <v>395</v>
+        <v>300</v>
       </c>
       <c r="U6" s="4">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="V6" s="3">
         <f>U6*12</f>
@@ -1453,13 +1484,13 @@
         <f>AA6-AB6-P6-Q6-R6-S6</f>
       </c>
       <c r="AE6" s="2">
-        <v>0.75</v>
+        <v>1.05</v>
       </c>
       <c r="AF6" s="1">
         <f>C6*AE6</f>
       </c>
       <c r="AG6" s="3">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="AH6" s="3">
         <f>V6*AG6*5</f>
@@ -1470,13 +1501,13 @@
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7" s="1">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
@@ -1494,10 +1525,10 @@
         <f>PMT(F7/12,G7*12,-E7)*12</f>
       </c>
       <c r="I7" s="1">
-        <v>2200</v>
+        <v>1400</v>
       </c>
       <c r="J7" s="1">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="K7" s="1">
         <v>1000</v>
@@ -1518,16 +1549,16 @@
         <f>(I7+J7)/3</f>
       </c>
       <c r="Q7" s="1">
-        <v>2200</v>
+        <v>1800</v>
       </c>
       <c r="R7" s="1">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="S7" s="1">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="T7" s="1">
-        <v>325</v>
+        <v>150</v>
       </c>
       <c r="U7" s="4">
         <v>15</v>
@@ -1560,13 +1591,13 @@
         <f>AA7-AB7-P7-Q7-R7-S7</f>
       </c>
       <c r="AE7" s="2">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="AF7" s="1">
         <f>C7*AE7</f>
       </c>
       <c r="AG7" s="3">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="AH7" s="3">
         <f>V7*AG7*5</f>
@@ -1577,13 +1608,13 @@
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C8" s="1">
-        <v>100000</v>
+        <v>32000</v>
       </c>
       <c r="D8" s="1">
         <v>0</v>
@@ -1625,16 +1656,16 @@
         <f>(I8+J8)/3</f>
       </c>
       <c r="Q8" s="1">
-        <v>2800</v>
+        <v>1800</v>
       </c>
       <c r="R8" s="1">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="S8" s="1">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="T8" s="1">
-        <v>425</v>
+        <v>120</v>
       </c>
       <c r="U8" s="4">
         <v>10</v>
@@ -1667,13 +1698,13 @@
         <f>AA8-AB8-P8-Q8-R8-S8</f>
       </c>
       <c r="AE8" s="2">
-        <v>0.68</v>
+        <v>0.85</v>
       </c>
       <c r="AF8" s="1">
         <f>C8*AE8</f>
       </c>
       <c r="AG8" s="3">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AH8" s="3">
         <f>V8*AG8*5</f>
@@ -1684,13 +1715,13 @@
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C9" s="1">
-        <v>55000</v>
+        <v>75000</v>
       </c>
       <c r="D9" s="1">
         <v>0</v>
@@ -1732,19 +1763,19 @@
         <f>(I9+J9)/3</f>
       </c>
       <c r="Q9" s="1">
-        <v>2200</v>
+        <v>2500</v>
       </c>
       <c r="R9" s="1">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="S9" s="1">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="T9" s="1">
-        <v>275</v>
+        <v>395</v>
       </c>
       <c r="U9" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="V9" s="3">
         <f>U9*12</f>
@@ -1774,13 +1805,13 @@
         <f>AA9-AB9-P9-Q9-R9-S9</f>
       </c>
       <c r="AE9" s="2">
-        <v>0.62</v>
+        <v>0.9</v>
       </c>
       <c r="AF9" s="1">
         <f>C9*AE9</f>
       </c>
       <c r="AG9" s="3">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AH9" s="3">
         <f>V9*AG9*5</f>
@@ -1791,13 +1822,13 @@
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C10" s="1">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="D10" s="1">
         <v>0</v>
@@ -1839,16 +1870,16 @@
         <f>(I10+J10)/3</f>
       </c>
       <c r="Q10" s="1">
-        <v>2000</v>
+        <v>2200</v>
       </c>
       <c r="R10" s="1">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="S10" s="1">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="T10" s="1">
-        <v>200</v>
+        <v>325</v>
       </c>
       <c r="U10" s="4">
         <v>15</v>
@@ -1881,13 +1912,13 @@
         <f>AA10-AB10-P10-Q10-R10-S10</f>
       </c>
       <c r="AE10" s="2">
-        <v>0.68</v>
+        <v>0.8</v>
       </c>
       <c r="AF10" s="1">
         <f>C10*AE10</f>
       </c>
       <c r="AG10" s="3">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="AH10" s="3">
         <f>V10*AG10*5</f>
@@ -1898,13 +1929,13 @@
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="1">
-        <v>45000</v>
+        <v>55000</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
@@ -1922,19 +1953,19 @@
         <f>PMT(F11/12,G11*12,-E11)*12</f>
       </c>
       <c r="I11" s="1">
-        <v>2200</v>
+        <v>1600</v>
       </c>
       <c r="J11" s="1">
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="K11" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L11" s="1">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="M11" s="1">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="N11" s="1">
         <f>SUM(I11:M11)</f>
@@ -1946,19 +1977,19 @@
         <f>(I11+J11)/3</f>
       </c>
       <c r="Q11" s="1">
-        <v>2000</v>
+        <v>2200</v>
       </c>
       <c r="R11" s="1">
-        <v>2800</v>
+        <v>3500</v>
       </c>
       <c r="S11" s="1">
         <v>1200</v>
       </c>
       <c r="T11" s="1">
-        <v>185</v>
+        <v>275</v>
       </c>
       <c r="U11" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="V11" s="3">
         <f>U11*12</f>
@@ -1967,10 +1998,10 @@
         <f>T11*V11</f>
       </c>
       <c r="X11" s="1">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="2">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="1">
         <f>V11*Y11*X11</f>
@@ -1988,13 +2019,13 @@
         <f>AA11-AB11-P11-Q11-R11-S11</f>
       </c>
       <c r="AE11" s="2">
-        <v>0.72</v>
+        <v>0.8</v>
       </c>
       <c r="AF11" s="1">
         <f>C11*AE11</f>
       </c>
       <c r="AG11" s="3">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="AH11" s="3">
         <f>V11*AG11*5</f>
@@ -2005,13 +2036,13 @@
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C12" s="1">
-        <v>85000</v>
+        <v>45000</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
@@ -2053,19 +2084,19 @@
         <f>(I12+J12)/3</f>
       </c>
       <c r="Q12" s="1">
-        <v>2300</v>
+        <v>2000</v>
       </c>
       <c r="R12" s="1">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="S12" s="1">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="T12" s="1">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="U12" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="V12" s="3">
         <f>U12*12</f>
@@ -2095,13 +2126,13 @@
         <f>AA12-AB12-P12-Q12-R12-S12</f>
       </c>
       <c r="AE12" s="2">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="AF12" s="1">
         <f>C12*AE12</f>
       </c>
       <c r="AG12" s="3">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="AH12" s="3">
         <f>V12*AG12*5</f>
@@ -2112,13 +2143,13 @@
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C13" s="1">
-        <v>70000</v>
+        <v>40000</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
@@ -2160,19 +2191,19 @@
         <f>(I13+J13)/3</f>
       </c>
       <c r="Q13" s="1">
-        <v>2200</v>
+        <v>2000</v>
       </c>
       <c r="R13" s="1">
-        <v>3200</v>
+        <v>2800</v>
       </c>
       <c r="S13" s="1">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="T13" s="1">
-        <v>325</v>
+        <v>185</v>
       </c>
       <c r="U13" s="4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="V13" s="3">
         <f>U13*12</f>
@@ -2202,13 +2233,13 @@
         <f>AA13-AB13-P13-Q13-R13-S13</f>
       </c>
       <c r="AE13" s="2">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="AF13" s="1">
         <f>C13*AE13</f>
       </c>
       <c r="AG13" s="3">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="AH13" s="3">
         <f>V13*AG13*5</f>
@@ -2219,13 +2250,13 @@
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="C14" s="1">
-        <v>52000</v>
+        <v>65000</v>
       </c>
       <c r="D14" s="1">
         <v>0</v>
@@ -2243,19 +2274,19 @@
         <f>PMT(F14/12,G14*12,-E14)*12</f>
       </c>
       <c r="I14" s="1">
+        <v>2200</v>
+      </c>
+      <c r="J14" s="1">
         <v>1600</v>
       </c>
-      <c r="J14" s="1">
-        <v>1400</v>
-      </c>
       <c r="K14" s="1">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="L14" s="1">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="M14" s="1">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="N14" s="1">
         <f>SUM(I14:M14)</f>
@@ -2267,19 +2298,19 @@
         <f>(I14+J14)/3</f>
       </c>
       <c r="Q14" s="1">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="R14" s="1">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="S14" s="1">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="T14" s="1">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="U14" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V14" s="3">
         <f>U14*12</f>
@@ -2288,10 +2319,10 @@
         <f>T14*V14</f>
       </c>
       <c r="X14" s="1">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="Y14" s="2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Z14" s="1">
         <f>V14*Y14*X14</f>
@@ -2309,13 +2340,13 @@
         <f>AA14-AB14-P14-Q14-R14-S14</f>
       </c>
       <c r="AE14" s="2">
-        <v>0.65</v>
+        <v>0.78</v>
       </c>
       <c r="AF14" s="1">
         <f>C14*AE14</f>
       </c>
       <c r="AG14" s="3">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="AH14" s="3">
         <f>V14*AG14*5</f>
@@ -2326,13 +2357,13 @@
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="C15" s="1">
-        <v>95000</v>
+        <v>75000</v>
       </c>
       <c r="D15" s="1">
         <v>0</v>
@@ -2374,16 +2405,16 @@
         <f>(I15+J15)/3</f>
       </c>
       <c r="Q15" s="1">
-        <v>2500</v>
+        <v>2200</v>
       </c>
       <c r="R15" s="1">
-        <v>4000</v>
+        <v>3200</v>
       </c>
       <c r="S15" s="1">
         <v>1500</v>
       </c>
       <c r="T15" s="1">
-        <v>475</v>
+        <v>325</v>
       </c>
       <c r="U15" s="4">
         <v>14</v>
@@ -2416,13 +2447,13 @@
         <f>AA15-AB15-P15-Q15-R15-S15</f>
       </c>
       <c r="AE15" s="2">
-        <v>0.72</v>
+        <v>0.8</v>
       </c>
       <c r="AF15" s="1">
         <f>C15*AE15</f>
       </c>
       <c r="AG15" s="3">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="AH15" s="3">
         <f>V15*AG15*5</f>
@@ -2433,13 +2464,13 @@
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C16" s="1">
-        <v>75000</v>
+        <v>80000</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
@@ -2481,19 +2512,19 @@
         <f>(I16+J16)/3</f>
       </c>
       <c r="Q16" s="1">
-        <v>2200</v>
+        <v>2500</v>
       </c>
       <c r="R16" s="1">
-        <v>3500</v>
+        <v>4000</v>
       </c>
       <c r="S16" s="1">
         <v>1500</v>
       </c>
       <c r="T16" s="1">
-        <v>325</v>
+        <v>475</v>
       </c>
       <c r="U16" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V16" s="3">
         <f>U16*12</f>
@@ -2529,7 +2560,7 @@
         <f>C16*AE16</f>
       </c>
       <c r="AG16" s="3">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="AH16" s="3">
         <f>V16*AG16*5</f>
@@ -2538,218 +2569,363 @@
         <f>AC16*5+AF16-D16</f>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" t="s">
+    <row r="17" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="1">
+      <c r="B17" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="13">
+        <f>SUM(C2:C16)</f>
+      </c>
+      <c r="D17" s="13">
+        <f>SUM(D2:D16)</f>
+      </c>
+      <c r="E17" s="13">
+        <f>SUM(E2:E16)</f>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="H17" s="13">
+        <f>SUM(H2:H16)</f>
+      </c>
+      <c r="I17" s="13">
+        <f>SUM(I2:I16)</f>
+      </c>
+      <c r="J17" s="13">
+        <f>SUM(J2:J16)</f>
+      </c>
+      <c r="K17" s="13">
+        <f>SUM(K2:K16)</f>
+      </c>
+      <c r="L17" s="13">
+        <f>SUM(L2:L16)</f>
+      </c>
+      <c r="M17" s="13">
+        <f>SUM(M2:M16)</f>
+      </c>
+      <c r="N17" s="13">
+        <f>SUM(N2:N16)</f>
+      </c>
+      <c r="O17" s="13">
+        <f>SUM(O2:O16)</f>
+      </c>
+      <c r="P17" s="13">
+        <f>SUM(P2:P16)</f>
+      </c>
+      <c r="Q17" s="13">
+        <f>SUM(Q2:Q16)</f>
+      </c>
+      <c r="R17" s="13">
+        <f>SUM(R2:R16)</f>
+      </c>
+      <c r="S17" s="13">
+        <f>SUM(S2:S16)</f>
+      </c>
+      <c r="T17" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="U17" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="V17" s="15">
+        <f>SUM(V2:V16)</f>
+      </c>
+      <c r="W17" s="13">
+        <f>SUM(W2:W16)</f>
+      </c>
+      <c r="X17" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y17" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z17" s="13">
+        <f>SUM(Z2:Z16)</f>
+      </c>
+      <c r="AA17" s="13">
+        <f>SUM(AA2:AA16)</f>
+      </c>
+      <c r="AB17" s="13">
+        <f>SUM(AB2:AB16)</f>
+      </c>
+      <c r="AC17" s="13">
+        <f>SUM(AC2:AC16)</f>
+      </c>
+      <c r="AD17" s="13">
+        <f>SUM(AD2:AD16)</f>
+      </c>
+      <c r="AE17" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF17" s="13">
+        <f>SUM(AF2:AF16)</f>
+      </c>
+      <c r="AG17" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH17" s="15">
+        <f>SUM(AH2:AH16)</f>
+      </c>
+      <c r="AI17" s="13">
+        <f>SUM(AI2:AI16)</f>
+      </c>
+    </row>
+    <row r="19" spans="1:35" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="19"/>
+      <c r="S19" s="19"/>
+      <c r="T19" s="19"/>
+      <c r="U19" s="22"/>
+      <c r="V19" s="21"/>
+      <c r="W19" s="19"/>
+      <c r="X19" s="19"/>
+      <c r="Y19" s="20"/>
+      <c r="Z19" s="19"/>
+      <c r="AA19" s="19"/>
+      <c r="AB19" s="19"/>
+      <c r="AC19" s="19"/>
+      <c r="AD19" s="19"/>
+      <c r="AE19" s="20"/>
+      <c r="AF19" s="19"/>
+      <c r="AG19" s="21"/>
+      <c r="AH19" s="21"/>
+      <c r="AI19" s="19"/>
+    </row>
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A20" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="24">
+        <v>60000</v>
+      </c>
+      <c r="D20" s="24">
+        <v>0</v>
+      </c>
+      <c r="E20" s="24">
+        <f>C20-D20</f>
+      </c>
+      <c r="F20" s="25">
+        <v>0.06</v>
+      </c>
+      <c r="G20" s="26">
+        <v>5</v>
+      </c>
+      <c r="H20" s="24">
+        <f>PMT(F20/12,G20*12,-E20)*12</f>
+      </c>
+      <c r="I20" s="24">
+        <v>2200</v>
+      </c>
+      <c r="J20" s="24">
+        <v>1600</v>
+      </c>
+      <c r="K20" s="24">
+        <v>1000</v>
+      </c>
+      <c r="L20" s="24">
+        <v>900</v>
+      </c>
+      <c r="M20" s="24">
+        <v>1500</v>
+      </c>
+      <c r="N20" s="24">
+        <f>SUM(I20:M20)</f>
+      </c>
+      <c r="O20" s="24">
+        <f>N20/G20</f>
+      </c>
+      <c r="P20" s="24">
+        <f>(I20+J20)/3</f>
+      </c>
+      <c r="Q20" s="24">
+        <v>2200</v>
+      </c>
+      <c r="R20" s="24">
+        <v>3500</v>
+      </c>
+      <c r="S20" s="24">
+        <v>1500</v>
+      </c>
+      <c r="T20" s="24">
+        <v>325</v>
+      </c>
+      <c r="U20" s="27">
+        <v>15</v>
+      </c>
+      <c r="V20" s="26">
+        <f>U20*12</f>
+      </c>
+      <c r="W20" s="24">
+        <f>T20*V20</f>
+      </c>
+      <c r="X20" s="24">
+        <v>35</v>
+      </c>
+      <c r="Y20" s="25">
+        <v>0.25</v>
+      </c>
+      <c r="Z20" s="24">
+        <f>V20*Y20*X20</f>
+      </c>
+      <c r="AA20" s="24">
+        <f>W20+Z20</f>
+      </c>
+      <c r="AB20" s="24">
+        <f>AA20*0.03</f>
+      </c>
+      <c r="AC20" s="24">
+        <f>AA20-AB20-H20-O20-P20-Q20-R20-S20</f>
+      </c>
+      <c r="AD20" s="24">
+        <f>AA20-AB20-P20-Q20-R20-S20</f>
+      </c>
+      <c r="AE20" s="25">
+        <v>0.72</v>
+      </c>
+      <c r="AF20" s="24">
+        <f>C20*AE20</f>
+      </c>
+      <c r="AG20" s="26">
+        <v>120</v>
+      </c>
+      <c r="AH20" s="26">
+        <f>V20*AG20*5</f>
+      </c>
+      <c r="AI20" s="24">
+        <f>AC20*5+AF20-D20</f>
+      </c>
+    </row>
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A21" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="24">
         <v>10000</v>
       </c>
-      <c r="D17" s="1">
-        <v>0</v>
-      </c>
-      <c r="E17" s="1">
-        <f>C17-D17</f>
-      </c>
-      <c r="F17" s="2">
+      <c r="D21" s="24">
+        <v>0</v>
+      </c>
+      <c r="E21" s="24">
+        <f>C21-D21</f>
+      </c>
+      <c r="F21" s="25">
         <v>0.06</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G21" s="26">
         <v>5</v>
       </c>
-      <c r="H17" s="1">
-        <f>PMT(F17/12,G17*12,-E17)*12</f>
-      </c>
-      <c r="I17" s="1">
+      <c r="H21" s="24">
+        <f>PMT(F21/12,G21*12,-E21)*12</f>
+      </c>
+      <c r="I21" s="24">
         <v>1400</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J21" s="24">
         <v>1000</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K21" s="24">
         <v>1000</v>
       </c>
-      <c r="L17" s="1">
+      <c r="L21" s="24">
         <v>900</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M21" s="24">
         <v>1500</v>
       </c>
-      <c r="N17" s="1">
-        <f>SUM(I17:M17)</f>
-      </c>
-      <c r="O17" s="1">
-        <f>N17/G17</f>
-      </c>
-      <c r="P17" s="1">
-        <f>(I17+J17)/3</f>
-      </c>
-      <c r="Q17" s="1">
+      <c r="N21" s="24">
+        <f>SUM(I21:M21)</f>
+      </c>
+      <c r="O21" s="24">
+        <f>N21/G21</f>
+      </c>
+      <c r="P21" s="24">
+        <f>(I21+J21)/3</f>
+      </c>
+      <c r="Q21" s="24">
         <v>1500</v>
       </c>
-      <c r="R17" s="1">
+      <c r="R21" s="24">
         <v>2500</v>
       </c>
-      <c r="S17" s="1">
+      <c r="S21" s="24">
         <v>1000</v>
       </c>
-      <c r="T17" s="1">
+      <c r="T21" s="24">
         <v>150</v>
       </c>
-      <c r="U17" s="4">
+      <c r="U21" s="27">
         <v>12.5</v>
       </c>
-      <c r="V17" s="3">
-        <f>U17*12</f>
-      </c>
-      <c r="W17" s="1">
-        <f>T17*V17</f>
-      </c>
-      <c r="X17" s="1">
+      <c r="V21" s="26">
+        <f>U21*12</f>
+      </c>
+      <c r="W21" s="24">
+        <f>T21*V21</f>
+      </c>
+      <c r="X21" s="24">
         <v>35</v>
       </c>
-      <c r="Y17" s="2">
+      <c r="Y21" s="25">
         <v>0.25</v>
       </c>
-      <c r="Z17" s="1">
-        <f>V17*Y17*X17</f>
-      </c>
-      <c r="AA17" s="1">
-        <f>W17+Z17</f>
-      </c>
-      <c r="AB17" s="1">
-        <f>AA17*0.03</f>
-      </c>
-      <c r="AC17" s="1">
-        <f>AA17-AB17-H17-O17-P17-Q17-R17-S17</f>
-      </c>
-      <c r="AD17" s="1">
-        <f>AA17-AB17-P17-Q17-R17-S17</f>
-      </c>
-      <c r="AE17" s="2">
+      <c r="Z21" s="24">
+        <f>V21*Y21*X21</f>
+      </c>
+      <c r="AA21" s="24">
+        <f>W21+Z21</f>
+      </c>
+      <c r="AB21" s="24">
+        <f>AA21*0.03</f>
+      </c>
+      <c r="AC21" s="24">
+        <f>AA21-AB21-H21-O21-P21-Q21-R21-S21</f>
+      </c>
+      <c r="AD21" s="24">
+        <f>AA21-AB21-P21-Q21-R21-S21</f>
+      </c>
+      <c r="AE21" s="25">
         <v>0.6</v>
       </c>
-      <c r="AF17" s="1">
-        <f>C17*AE17</f>
-      </c>
-      <c r="AG17" s="3">
+      <c r="AF21" s="24">
+        <f>C21*AE21</f>
+      </c>
+      <c r="AG21" s="26">
         <v>130</v>
       </c>
-      <c r="AH17" s="3">
-        <f>V17*AG17*5</f>
-      </c>
-      <c r="AI17" s="1">
-        <f>AC17*5+AF17-D17</f>
-      </c>
-    </row>
-    <row r="18" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" s="13">
-        <f>SUM(C2:C17)</f>
-      </c>
-      <c r="D18" s="13">
-        <f>SUM(D2:D17)</f>
-      </c>
-      <c r="E18" s="13">
-        <f>SUM(E2:E17)</f>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="G18" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="H18" s="13">
-        <f>SUM(H2:H17)</f>
-      </c>
-      <c r="I18" s="13">
-        <f>SUM(I2:I17)</f>
-      </c>
-      <c r="J18" s="13">
-        <f>SUM(J2:J17)</f>
-      </c>
-      <c r="K18" s="13">
-        <f>SUM(K2:K17)</f>
-      </c>
-      <c r="L18" s="13">
-        <f>SUM(L2:L17)</f>
-      </c>
-      <c r="M18" s="13">
-        <f>SUM(M2:M17)</f>
-      </c>
-      <c r="N18" s="13">
-        <f>SUM(N2:N17)</f>
-      </c>
-      <c r="O18" s="13">
-        <f>SUM(O2:O17)</f>
-      </c>
-      <c r="P18" s="13">
-        <f>SUM(P2:P17)</f>
-      </c>
-      <c r="Q18" s="13">
-        <f>SUM(Q2:Q17)</f>
-      </c>
-      <c r="R18" s="13">
-        <f>SUM(R2:R17)</f>
-      </c>
-      <c r="S18" s="13">
-        <f>SUM(S2:S17)</f>
-      </c>
-      <c r="T18" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="U18" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="V18" s="15">
-        <f>SUM(V2:V17)</f>
-      </c>
-      <c r="W18" s="13">
-        <f>SUM(W2:W17)</f>
-      </c>
-      <c r="X18" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y18" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="Z18" s="13">
-        <f>SUM(Z2:Z17)</f>
-      </c>
-      <c r="AA18" s="13">
-        <f>SUM(AA2:AA17)</f>
-      </c>
-      <c r="AB18" s="13">
-        <f>SUM(AB2:AB17)</f>
-      </c>
-      <c r="AC18" s="13">
-        <f>SUM(AC2:AC17)</f>
-      </c>
-      <c r="AD18" s="13">
-        <f>SUM(AD2:AD17)</f>
-      </c>
-      <c r="AE18" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="AF18" s="13">
-        <f>SUM(AF2:AF17)</f>
-      </c>
-      <c r="AG18" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="AH18" s="15">
-        <f>SUM(AH2:AH17)</f>
-      </c>
-      <c r="AI18" s="13">
-        <f>SUM(AI2:AI17)</f>
+      <c r="AH21" s="26">
+        <f>V21*AG21*5</f>
+      </c>
+      <c r="AI21" s="24">
+        <f>AC21*5+AF21-D21</f>
       </c>
     </row>
   </sheetData>
@@ -2767,164 +2943,164 @@
     <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" s="17" t="s">
-        <v>65</v>
+    <row r="1" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B3" s="1">
-        <f>SUM('Fleet Model'!C2:C17)</f>
+        <f>SUM('Fleet Model'!C2:C16)</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B4" s="1">
-        <f>SUM('Fleet Model'!N2:N17)</f>
+        <f>SUM('Fleet Model'!N2:N16)</f>
       </c>
     </row>
     <row r="5" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="18">
-        <f>SUM('Fleet Model'!C2:C17)+SUM('Fleet Model'!N2:N17)</f>
+        <v>73</v>
+      </c>
+      <c r="B5" s="29">
+        <f>SUM('Fleet Model'!C2:C16)+SUM('Fleet Model'!N2:N16)</f>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B7" s="1">
-        <f>SUM('Fleet Model'!W2:W17)</f>
+        <f>SUM('Fleet Model'!W2:W16)</f>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B8" s="1">
-        <f>SUM('Fleet Model'!Z2:Z17)</f>
+        <f>SUM('Fleet Model'!Z2:Z16)</f>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B9" s="1">
-        <f>SUM('Fleet Model'!AA2:AA17)</f>
+        <f>SUM('Fleet Model'!AA2:AA16)</f>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B10" s="1">
-        <f>SUM('Fleet Model'!AB2:AB17)</f>
+        <f>SUM('Fleet Model'!AB2:AB16)</f>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B11" s="1">
-        <f>SUM('Fleet Model'!P2:P17)</f>
+        <f>SUM('Fleet Model'!P2:P16)</f>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B12" s="1">
-        <f>SUM('Fleet Model'!AC2:AC17)</f>
+        <f>SUM('Fleet Model'!AC2:AC16)</f>
       </c>
     </row>
     <row r="13" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="18">
-        <f>SUM('Fleet Model'!AD2:AD17)</f>
+        <v>80</v>
+      </c>
+      <c r="B13" s="29">
+        <f>SUM('Fleet Model'!AD2:AD16)</f>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B15" s="1">
-        <f>SUM('Fleet Model'!AF2:AF17)</f>
+        <f>SUM('Fleet Model'!AF2:AF16)</f>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B16" s="3">
-        <f>SUM('Fleet Model'!AH2:AH17)</f>
+        <f>SUM('Fleet Model'!AH2:AH16)</f>
       </c>
     </row>
     <row r="17" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B17" s="18">
-        <f>SUM('Fleet Model'!AI2:AI17)</f>
+        <v>83</v>
+      </c>
+      <c r="B17" s="29">
+        <f>SUM('Fleet Model'!AI2:AI16)</f>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B19" s="1">
-        <f>SUM('Fleet Model'!AC2:AC17)/16</f>
+        <f>SUM('Fleet Model'!AC2:AC16)/15</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B20" s="19">
-        <f>SUM('Fleet Model'!AI2:AI17)/(SUM('Fleet Model'!C2:C17)+SUM('Fleet Model'!N2:N17))</f>
+        <v>85</v>
+      </c>
+      <c r="B20" s="30">
+        <f>SUM('Fleet Model'!AI2:AI16)/(SUM('Fleet Model'!C2:C16)+SUM('Fleet Model'!N2:N16))</f>
       </c>
     </row>
   </sheetData>
@@ -2935,243 +3111,235 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="62" style="20" customWidth="1"/>
+    <col min="2" max="2" width="62" style="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="22" t="s">
-        <v>65</v>
+    <row r="1" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>84</v>
+        <v>87</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>86</v>
+        <v>89</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>88</v>
+        <v>91</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>65</v>
+        <v>93</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>91</v>
+        <v>64</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>93</v>
+        <v>96</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>95</v>
+        <v>64</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>65</v>
+        <v>99</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>65</v>
+        <v>101</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>99</v>
+        <v>103</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>100</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>101</v>
+        <v>105</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>103</v>
+        <v>15</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>105</v>
+        <v>64</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>65</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>107</v>
+        <v>25</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="32" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" s="33" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="20" t="s">
-        <v>108</v>
+      <c r="B23" s="31" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="20" t="s">
-        <v>109</v>
+      <c r="B24" s="31" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="20" t="s">
-        <v>110</v>
+      <c r="B25" s="31" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>65</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="B26" s="31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="B27" s="33" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>112</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>114</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>115</v>
+        <v>116</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>